<commit_message>
video 31 đến 46
</commit_message>
<xml_diff>
--- a/steps.xlsx
+++ b/steps.xlsx
@@ -19,10 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>video 21</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t xml:space="preserve"> phân loại sản phẩm theo danh mục</t>
   </si>
@@ -345,7 +342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.109375" customWidth="1"/>
@@ -353,14 +350,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>